<commit_message>
fix: plantilla carga masiva — agregar columnas de conyuge y ejemplo MATRIMONIO
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/front/public/templates/plantilla_carga_masiva.xlsx
+++ b/front/public/templates/plantilla_carga_masiva.xlsx
@@ -397,7 +397,34 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:Y5"/>
+  <cols>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="8.83203125" customWidth="1"/>
+    <col min="4" max="4" width="13.83203125" customWidth="1"/>
+    <col min="5" max="5" width="6.83203125" customWidth="1"/>
+    <col min="6" max="6" width="13.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" customWidth="1"/>
+    <col min="9" max="9" width="20.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="18.83203125" customWidth="1"/>
+    <col min="12" max="12" width="6.83203125" customWidth="1"/>
+    <col min="13" max="13" width="15.83203125" customWidth="1"/>
+    <col min="14" max="14" width="13.83203125" customWidth="1"/>
+    <col min="15" max="15" width="22.83203125" customWidth="1"/>
+    <col min="16" max="16" width="16.83203125" customWidth="1"/>
+    <col min="17" max="17" width="20.83203125" customWidth="1"/>
+    <col min="18" max="18" width="20.83203125" customWidth="1"/>
+    <col min="19" max="19" width="20.83203125" customWidth="1"/>
+    <col min="20" max="20" width="20.83203125" customWidth="1"/>
+    <col min="21" max="21" width="13.83203125" customWidth="1"/>
+    <col min="22" max="22" width="22.83203125" customWidth="1"/>
+    <col min="23" max="23" width="25.83203125" customWidth="1"/>
+    <col min="24" max="24" width="20.83203125" customWidth="1"/>
+    <col min="25" max="25" width="22.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -443,16 +470,37 @@
         <v>telefono</v>
       </c>
       <c r="O1" t="str">
+        <v>persona_observaciones</v>
+      </c>
+      <c r="P1" t="str">
+        <v>conyuge_dni</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>conyuge_tipo_documento</v>
+      </c>
+      <c r="R1" t="str">
+        <v>conyuge_nombres</v>
+      </c>
+      <c r="S1" t="str">
+        <v>conyuge_apellido_paterno</v>
+      </c>
+      <c r="T1" t="str">
+        <v>conyuge_apellido_materno</v>
+      </c>
+      <c r="U1" t="str">
+        <v>conyuge_sexo</v>
+      </c>
+      <c r="V1" t="str">
+        <v>conyuge_fecha_nacimiento</v>
+      </c>
+      <c r="W1" t="str">
+        <v>nombre_archivo_pdf</v>
+      </c>
+      <c r="X1" t="str">
+        <v>carpeta_ruta</v>
+      </c>
+      <c r="Y1" t="str">
         <v>acta_observaciones</v>
-      </c>
-      <c r="P1" t="str">
-        <v>persona_observaciones</v>
-      </c>
-      <c r="Q1" t="str">
-        <v>nombre_archivo_pdf</v>
-      </c>
-      <c r="R1" t="str">
-        <v>carpeta_ruta</v>
       </c>
     </row>
     <row r="2">
@@ -460,7 +508,7 @@
         <v>NACIMIENTO</v>
       </c>
       <c r="B2" t="str">
-        <v>12345678</v>
+        <v>20241234567890</v>
       </c>
       <c r="C2" t="str">
         <v/>
@@ -493,21 +541,42 @@
         <v>M</v>
       </c>
       <c r="M2" t="str">
-        <v>2024-01-01</v>
+        <v>2000-05-15</v>
       </c>
       <c r="N2" t="str">
         <v>987654321</v>
       </c>
       <c r="O2" t="str">
-        <v>Registro masivo CUI</v>
+        <v/>
       </c>
       <c r="P2" t="str">
         <v/>
       </c>
       <c r="Q2" t="str">
-        <v>ejemplo_cui.pdf</v>
+        <v/>
       </c>
       <c r="R2" t="str">
+        <v/>
+      </c>
+      <c r="S2" t="str">
+        <v/>
+      </c>
+      <c r="T2" t="str">
+        <v/>
+      </c>
+      <c r="U2" t="str">
+        <v/>
+      </c>
+      <c r="V2" t="str">
+        <v/>
+      </c>
+      <c r="W2" t="str">
+        <v>nacimiento_001.pdf</v>
+      </c>
+      <c r="X2" t="str">
+        <v/>
+      </c>
+      <c r="Y2" t="str">
         <v/>
       </c>
     </row>
@@ -555,21 +624,196 @@
         <v/>
       </c>
       <c r="O3" t="str">
-        <v>Registro masivo Clásico</v>
+        <v/>
       </c>
       <c r="P3" t="str">
         <v/>
       </c>
       <c r="Q3" t="str">
-        <v>ejemplo_libro.pdf</v>
+        <v/>
       </c>
       <c r="R3" t="str">
-        <v>actas/1995</v>
+        <v/>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str">
+        <v/>
+      </c>
+      <c r="V3" t="str">
+        <v/>
+      </c>
+      <c r="W3" t="str">
+        <v>nac_libro45_123.pdf</v>
+      </c>
+      <c r="X3" t="str">
+        <v>nacimientos/1995</v>
+      </c>
+      <c r="Y3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>MATRIMONIO</v>
+      </c>
+      <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
+        <v>12</v>
+      </c>
+      <c r="D4" t="str">
+        <v>55</v>
+      </c>
+      <c r="E4">
+        <v>2023</v>
+      </c>
+      <c r="F4" t="str">
+        <v>2023-08-20</v>
+      </c>
+      <c r="G4" t="str">
+        <v>45678901</v>
+      </c>
+      <c r="H4" t="str">
+        <v>DNI</v>
+      </c>
+      <c r="I4" t="str">
+        <v>CARLOS MIGUEL</v>
+      </c>
+      <c r="J4" t="str">
+        <v>TORRES</v>
+      </c>
+      <c r="K4" t="str">
+        <v>QUISPE</v>
+      </c>
+      <c r="L4" t="str">
+        <v>M</v>
+      </c>
+      <c r="M4" t="str">
+        <v>1990-03-10</v>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
+        <v>56789012</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>DNI</v>
+      </c>
+      <c r="R4" t="str">
+        <v>ANA LUCIA</v>
+      </c>
+      <c r="S4" t="str">
+        <v>MAMANI</v>
+      </c>
+      <c r="T4" t="str">
+        <v>FLORES</v>
+      </c>
+      <c r="U4" t="str">
+        <v>F</v>
+      </c>
+      <c r="V4" t="str">
+        <v>1992-07-22</v>
+      </c>
+      <c r="W4" t="str">
+        <v>matrimonio_55.pdf</v>
+      </c>
+      <c r="X4" t="str">
+        <v>matrimonios/2023</v>
+      </c>
+      <c r="Y4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>DEFUNCION</v>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v>8</v>
+      </c>
+      <c r="D5" t="str">
+        <v>201</v>
+      </c>
+      <c r="E5">
+        <v>2022</v>
+      </c>
+      <c r="F5" t="str">
+        <v>2022-11-05</v>
+      </c>
+      <c r="G5" t="str">
+        <v>11223344</v>
+      </c>
+      <c r="H5" t="str">
+        <v>DNI</v>
+      </c>
+      <c r="I5" t="str">
+        <v>PEDRO JOSE</v>
+      </c>
+      <c r="J5" t="str">
+        <v>VARGAS</v>
+      </c>
+      <c r="K5" t="str">
+        <v>HUANCA</v>
+      </c>
+      <c r="L5" t="str">
+        <v>M</v>
+      </c>
+      <c r="M5" t="str">
+        <v>1945-01-30</v>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+      <c r="O5" t="str">
+        <v/>
+      </c>
+      <c r="P5" t="str">
+        <v/>
+      </c>
+      <c r="Q5" t="str">
+        <v/>
+      </c>
+      <c r="R5" t="str">
+        <v/>
+      </c>
+      <c r="S5" t="str">
+        <v/>
+      </c>
+      <c r="T5" t="str">
+        <v/>
+      </c>
+      <c r="U5" t="str">
+        <v/>
+      </c>
+      <c r="V5" t="str">
+        <v/>
+      </c>
+      <c r="W5" t="str">
+        <v>defuncion_201.pdf</v>
+      </c>
+      <c r="X5" t="str">
+        <v>defunciones/2022</v>
+      </c>
+      <c r="Y5" t="str">
+        <v>Fallecimiento natural</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Y5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>